<commit_message>
Refine mappings in CdaIVL-TSToPeriodConceptMap
Updated descriptions and mappings for CDA IVL_TS to FHIR Period and dateTime. e11bd07ca4806222b80177a02e2c6d998a83ff4c
</commit_message>
<xml_diff>
--- a/traitement-erreur/ig/CdaIVL-TSToPeriodConceptMap.xlsx
+++ b/traitement-erreur/ig/CdaIVL-TSToPeriodConceptMap.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="61" uniqueCount="40">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="61" uniqueCount="47">
   <si>
     <t>Property</t>
   </si>
@@ -25,7 +25,7 @@
     <t>URL</t>
   </si>
   <si>
-    <t>https://interop.esante.gouv.fr/ig/fhir/mappingcdafhir/ConceptMap/DataTypes/CdaIVL_TSToFHIR</t>
+    <t>https://interop.esante.gouv.fr/ig/fhir/mappingcdafhir/ConceptMap/CdaIVL-TSToPeriodConceptMap</t>
   </si>
   <si>
     <t>Version</t>
@@ -61,7 +61,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-07-22T13:17:03+00:00</t>
+    <t>2026-07-22T13:34:22+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -85,7 +85,7 @@
     <t>Description</t>
   </si>
   <si>
-    <t>Correspondances documentaires entre le datatype CDA IVL_TS et les types FHIR Period et dateTime.</t>
+    <t>Correspondances documentaires entre le datatype CDA IVL_TS, ses bornes IVXB_TS et les types FHIR Period et dateTime.</t>
   </si>
   <si>
     <t>Purpose</t>
@@ -115,7 +115,10 @@
     <t>http://hl7.org/fhir/StructureDefinition/Period|4.0.1</t>
   </si>
   <si>
-    <t>IVL_TS.low.value</t>
+    <t>IVL_TS.low</t>
+  </si>
+  <si>
+    <t>Low Boundary</t>
   </si>
   <si>
     <t>related-to</t>
@@ -124,16 +127,34 @@
     <t>Period.start</t>
   </si>
   <si>
-    <t>IVL_TS.high.value</t>
+    <t>Starting time with inclusive boundary</t>
+  </si>
+  <si>
+    <t>IVL_TS.high</t>
+  </si>
+  <si>
+    <t>High Boundary</t>
   </si>
   <si>
     <t>Period.end</t>
   </si>
   <si>
+    <t>End time with inclusive boundary, if not ongoing</t>
+  </si>
+  <si>
+    <t>http://hl7.org/cda/stds/core/StructureDefinition/IVXB-TS|2.0.0-sd</t>
+  </si>
+  <si>
     <t>http://hl7.org/fhir/StructureDefinition/dateTime|4.0.1</t>
   </si>
   <si>
+    <t>IVXB_TS.value</t>
+  </si>
+  <si>
     <t>dateTime</t>
+  </si>
+  <si>
+    <t>Primitive Type dateTime</t>
   </si>
 </sst>
 </file>
@@ -431,33 +452,33 @@
         <v>33</v>
       </c>
       <c r="B3" t="s" s="2">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="C3" t="s" s="2">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="D3" t="s" s="2">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="E3" t="s" s="2">
-        <v>35</v>
+        <v>37</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s" s="2">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="B4" t="s" s="2">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="C4" t="s" s="2">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="D4" t="s" s="2">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="E4" t="s" s="2">
-        <v>37</v>
+        <v>41</v>
       </c>
     </row>
   </sheetData>
@@ -489,7 +510,7 @@
     </row>
     <row r="2">
       <c r="A2" t="s" s="2">
-        <v>30</v>
+        <v>42</v>
       </c>
       <c r="B2" t="s" s="2">
         <v>31</v>
@@ -498,7 +519,7 @@
         <v>31</v>
       </c>
       <c r="D2" t="s" s="2">
-        <v>38</v>
+        <v>43</v>
       </c>
       <c r="E2" t="s" s="2">
         <v>31</v>
@@ -506,19 +527,19 @@
     </row>
     <row r="3">
       <c r="A3" t="s" s="2">
-        <v>33</v>
+        <v>44</v>
       </c>
       <c r="B3" t="s" s="2">
-        <v>33</v>
+        <v>44</v>
       </c>
       <c r="C3" t="s" s="2">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="D3" t="s" s="2">
-        <v>39</v>
+        <v>45</v>
       </c>
       <c r="E3" t="s" s="2">
-        <v>39</v>
+        <v>46</v>
       </c>
     </row>
   </sheetData>

</xml_diff>